<commit_message>
Expand legal terms library to 105 terms
- Updated create_legal_library.py with 95 additional legal terms
- Legal terms now range from LT001 to LT105
- Comprehensive coverage of criminal, civil, and procedural law terms
- Regenerated legal_terms_library.xlsx with all 105 terms
</commit_message>
<xml_diff>
--- a/legal_terms_library.xlsx
+++ b/legal_terms_library.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -685,6 +685,2096 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>LT011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Brief</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>A written statement submitted by the lawyer for each side in a case that explains the law and facts supporting that party's case</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>LT012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Burden of Proof</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>The duty to prove disputed facts in a case resting on the party asserting the affirmative of an issue</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>LT013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Case Law</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Law established by previous decisions of appellate courts particularly the Supreme Court</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>LT014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Chambers</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>The offices of a judge and the judge's staff</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>LT015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Change of Venue</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Moving a lawsuit or criminal trial to another place for trial</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>LT016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Civil Action</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>A lawsuit brought to enforce protect or redress private or civil rights</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>LT017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Class Action</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>A lawsuit in which one or more members of a large group represent the entire group</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>LT018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Clerk of Court</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>An officer appointed by the court to work with the chief judge in overseeing the court's administration</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>LT019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Common Law</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>The legal system that originated in England and is now in use in the United States based on judicial decisions</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>LT020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Complaint</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>A written statement that begins a civil lawsuit containing the plaintiff's allegations against the defendant</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>LT021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Concurrent Sentence</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Prison terms for two or more offenses to be served at the same time rather than consecutively</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>LT022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Consecutive Sentence</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Prison terms for two or more offenses to be served one after the other</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>LT023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>An agreement between two or more persons that creates an obligation to do or not to do a particular thing</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>LT024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Conviction</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>A judgment of guilt against a criminal defendant</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>LT025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Court Reporter</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>A person who makes a word-for-word record of what is said in court and produces a transcript upon request</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>LT026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Creditor</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>A person to whom money is owed by another person called the debtor</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>LT027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Cross-Examination</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Questioning of a witness by the opposing party during a trial or deposition</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>LT028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Damages</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Money paid by defendants to successful plaintiffs in civil cases to compensate the plaintiffs for their injuries</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>LT029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Debtor</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>A person who owes money to a creditor</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>LT030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Declaratory Judgment</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>A judge's statement about someone's rights without ordering that anything be done</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>LT031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Default Judgment</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>A judgment rendered because of the defendant's failure to answer or appear in court</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>LT032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Defendant</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>The person or entity defending against a lawsuit or criminal prosecution</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>LT033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Deposition</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>An oral statement made before an officer authorized by law to administer oaths taken before trial</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>LT034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>The pretrial process by which parties gather information from each other</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>LT035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Dismissal</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>An order or judgment disposing of a case without a trial</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>LT036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Docket</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>A log containing the complete history of each case in the form of brief chronological entries</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>LT037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Due Process</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>The right to a fair and impartial hearing including notice of charges and opportunity to be heard</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>LT038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>En Banc</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>A proceeding in which the entire court participates in the decision rather than a subset of judges</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>LT039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Information presented in testimony or in documents used to persuade the fact finder</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>LT040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Executor</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>A personal representative named in a will to administer the estate of a deceased person</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>LT041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Exempt Assets</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Property that a debtor is allowed to retain free from the claims of creditors</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>LT042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Expert Witness</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>A witness with specialized knowledge or training who testifies about professional or scientific matters</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>LT043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Felony</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>A serious crime usually punishable by imprisonment for more than one year or death</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>LT044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Filing</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>The act of submitting a document to the court clerk for inclusion in the case file</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>LT045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Foreclosure</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>A legal proceeding to terminate a property owner's rights in property</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>LT046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Fraudulent Transfer</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>A transfer of a debtor's property made with intent to defraud creditors</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>LT047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Grand Jury</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>A body of citizens who listen to evidence and determine whether there is probable cause to believe a crime was committed</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>LT048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Habeas Corpus</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>A writ that is usually used to bring a prisoner before the court to determine the legality of imprisonment</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>LT049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Hearsay</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Evidence presented by a witness based on what others have said rather than personal knowledge</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>LT050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Impeachment</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>The process of calling something into question such as the testimony of a witness</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>LT051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>In Camera</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>In chambers or in private where the public and jury are excluded</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>LT052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Indictment</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>The formal charge issued by a grand jury stating there is enough evidence to require a trial</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>LT053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Injunction</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>A court order preventing one or more named parties from taking some action</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>LT054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Interrogatories</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Written questions developed by one party and sent to another party to be answered under oath</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>LT055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Joint Administration</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>A court-approved mechanism under which two or more cases can be administered together</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>LT056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>The official decision of a court finally determining the respective rights and claims of the parties</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>LT057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Jurisdiction</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>The legal authority of a court to hear and decide a case</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>LT058</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Jury</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>A group of citizens who hear the evidence presented by both sides at trial and determine the facts in dispute</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>LT059</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Jury Instructions</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>A judge's directions to the jury before it begins deliberations regarding the law that applies to the case</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>LT060</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Lien</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>A charge or claim on property as security for a debt or obligation</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>LT061</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Litigation</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>A case lawsuit or action in a civil or criminal court</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>LT062</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Magistrate Judge</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>A judicial officer who assists district court judges in preparing cases for trial</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>LT063</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Malpractice</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Professional misconduct or unreasonable lack of skill by a professional</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>LT064</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Mandamus</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>A writ issued by a court ordering a public official to perform an act</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>LT065</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Material Witness</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>A witness whose testimony is essential to a case</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>LT066</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Mediation</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>A form of alternative dispute resolution in which a neutral third party assists in resolving a dispute</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>LT067</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Misdemeanor</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>A crime less serious than a felony usually punishable by fine or imprisonment for less than one year</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>LT068</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Mistrial</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>An invalid trial caused by fundamental error resulting in termination of trial before a verdict</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>LT069</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>A request by a litigant asking the court to decide an issue in the case</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>LT070</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Motion in Limine</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>A pretrial motion requesting the court to prohibit the opposing party from referring to certain matters</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>LT071</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Negligence</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Failure to exercise the degree of care that a reasonable person would exercise under the same circumstances</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>LT072</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Nolo Contendere</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>No contest - a plea by which a defendant does not expressly admit guilt</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>LT073</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Notary Public</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>A public officer authorized to administer oaths and certify documents</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>LT074</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Oath</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>A solemn pledge made under a sense of responsibility in attestation of truth of a statement</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>LT075</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Objection</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>A protest by an attorney challenging a statement or question made at trial</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>LT076</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Opinion</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>A judge's written explanation of a decision or judgment</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>LT077</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Oral Argument</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>An opportunity for lawyers to summarize their position before the court and answer questions</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>LT078</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>A written command or direction issued by a judge</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>LT079</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Ordinance</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>A law passed by a local government such as a city or county</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>LT080</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Parole</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>The supervised release of a prisoner before completion of the full sentence</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>LT081</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>A person business or government agency actively involved in the prosecution or defense of a legal proceeding</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>LT082</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Perjury</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>The criminal offense of making false statements under oath</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>LT083</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Petition</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>A formal written request asking the court for specific relief</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>LT084</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Petitioner</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>The party filing a petition especially an appeal</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>LT085</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Plaintiff</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>The person who files the complaint in a civil lawsuit</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>LT086</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Plea</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>In a criminal proceeding the defendant's declaration in open court of guilt or innocence</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>LT087</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Plea Bargain</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>An agreement between the prosecutor and defendant where the defendant pleads guilty in exchange for concessions</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>LT088</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Pleadings</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Written statements of the parties in a civil case detailing their claims defenses and replies</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>LT089</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Precedent</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>A court decision in an earlier case with facts and law similar to a dispute currently before a court</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>LT090</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Preliminary Injunction</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>A court order to preserve the status quo until a hearing can be held</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>LT091</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Preponderance of Evidence</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>The greater weight of the evidence required in most civil cases</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>LT092</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Presentence Report</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>A report prepared by a probation officer after conviction to assist the judge in sentencing</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>LT093</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Pretrial Conference</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>A meeting between the judge and lawyers to narrow issues prepare for trial and explore settlement</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>LT094</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Probation</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>A sentencing alternative allowing a convicted defendant to serve their sentence outside of jail under supervision</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>LT095</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Pro Se</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Representing oneself without an attorney in a legal proceeding</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>LT096</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Prosecutor</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>A government attorney who presents the state's case against a defendant in a criminal proceeding</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>LT097</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Quash</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>To nullify void or declare invalid such as quashing a subpoena</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>LT098</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Reasonable Doubt</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>The level of certainty a juror must have to find a defendant guilty of a crime</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>LT099</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Rebuttal</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Evidence offered to contradict or disprove evidence presented by the opposing party</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>LT100</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>A written account of all the proceedings in a case including all pleadings evidence and exhibits</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>LT101</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Remand</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>When an appellate court sends a case back to a lower court for further proceedings</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>LT102</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Respondent</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>The party against whom an appeal or motion is filed</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>LT103</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Restitution</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>The act of compensating someone for loss damage or injury by the party responsible</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>LT104</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Retainer</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>An advance payment to an attorney for legal services to be rendered</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>DOJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>LT105</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Sanction</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>A penalty or other enforcement measure used to provide incentives for compliance with the law</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>US Courts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>